<commit_message>
:recycle: Refactor export pipeline
</commit_message>
<xml_diff>
--- a/examples/template.xlsx
+++ b/examples/template.xlsx
@@ -105,7 +105,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -240,11 +240,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom style="thin">
+        <color rgb="FF94A3B8"/>
+      </bottom>
+    </border>
+    <border>
+      <right/>
+      <bottom style="medium">
+        <color rgb="FF17324D"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -298,6 +310,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -677,32 +697,32 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>{{report_title:string}}</t>
         </is>
       </c>
-      <c r="B1" s="13" t="n"/>
-      <c r="C1" s="13" t="n"/>
-      <c r="D1" s="13" t="n"/>
-      <c r="E1" s="13" t="n"/>
-      <c r="F1" s="13" t="n"/>
-      <c r="G1" s="13" t="n"/>
-      <c r="H1" s="13" t="n"/>
+      <c r="B1" s="24" t="n"/>
+      <c r="C1" s="24" t="n"/>
+      <c r="D1" s="24" t="n"/>
+      <c r="E1" s="24" t="n"/>
+      <c r="F1" s="24" t="n"/>
+      <c r="G1" s="24" t="n"/>
+      <c r="H1" s="24" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="25" t="inlineStr">
         <is>
           <t>{{status:string}}</t>
         </is>
       </c>
-      <c r="B2" s="15" t="n"/>
-      <c r="C2" s="15" t="n"/>
-      <c r="D2" s="15" t="n"/>
-      <c r="E2" s="15" t="n"/>
-      <c r="F2" s="15" t="n"/>
-      <c r="G2" s="15" t="n"/>
-      <c r="H2" s="15" t="n"/>
+      <c r="B2" s="26" t="n"/>
+      <c r="C2" s="26" t="n"/>
+      <c r="D2" s="26" t="n"/>
+      <c r="E2" s="26" t="n"/>
+      <c r="F2" s="26" t="n"/>
+      <c r="G2" s="26" t="n"/>
+      <c r="H2" s="26" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -754,7 +774,7 @@
     <row r="8" ht="25" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>{{line_item_headers:dataframe-headers}}</t>
+          <t>{{line_item_headers:dataframe-header}}</t>
         </is>
       </c>
     </row>

</xml_diff>